<commit_message>
Entrega 2b · primera carga real de la alfa
TSK fijado como TSK.MC; el proyector excluye series sin cotizacion reciente (>30 dias) y
normaliza los gastos corrientes de EODHD a porcentaje; gcloud.cmd con shell en Windows.
Carga publicada en nuvia-family-wealth: 159 activos, 932 series, 7 desgloses, datos hasta
2026-09-02; excluidos LU2267099674 (sin precios) y ES0143416115 (sin cotizacion desde 2023).
Estado de la entrega en docs/ESTADO_ENTREGA_2B_20260902.md.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVE8DgVshCWowUtq2RoFmT
</commit_message>
<xml_diff>
--- a/universo/universo-alfa.xlsx
+++ b/universo/universo-alfa.xlsx
@@ -30674,7 +30674,11 @@
           <t>ES0105394003</t>
         </is>
       </c>
-      <c r="B720" t="inlineStr"/>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>TSK.MC</t>
+        </is>
+      </c>
       <c r="C720" t="inlineStr">
         <is>
           <t>STOCK</t>

</xml_diff>